<commit_message>
feat(ai): merge 2500 sample and 18901 reviews into final master emotion lexicon codebook
</commit_message>
<xml_diff>
--- a/data/derived_outputs/gold_emotion_lexicon_codebook.xlsx
+++ b/data/derived_outputs/gold_emotion_lexicon_codebook.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4265" uniqueCount="1743">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4265" uniqueCount="1742">
   <si>
     <t>word</t>
   </si>
@@ -1477,222 +1477,222 @@
     <t>apprehension</t>
   </si>
   <si>
+    <t>comforted</t>
+  </si>
+  <si>
+    <t>envy</t>
+  </si>
+  <si>
+    <t>faultless</t>
+  </si>
+  <si>
+    <t>gloomy</t>
+  </si>
+  <si>
+    <t>hated</t>
+  </si>
+  <si>
+    <t>hates</t>
+  </si>
+  <si>
+    <t>intimidating</t>
+  </si>
+  <si>
+    <t>jitters</t>
+  </si>
+  <si>
+    <t>joyful</t>
+  </si>
+  <si>
+    <t>luscious</t>
+  </si>
+  <si>
+    <t>marveled</t>
+  </si>
+  <si>
+    <t>nauseated</t>
+  </si>
+  <si>
+    <t>overwhelmingly</t>
+  </si>
+  <si>
+    <t>pity</t>
+  </si>
+  <si>
+    <t>scare</t>
+  </si>
+  <si>
+    <t>shock</t>
+  </si>
+  <si>
+    <t>stressful</t>
+  </si>
+  <si>
+    <t>suprise</t>
+  </si>
+  <si>
+    <t>wowed</t>
+  </si>
+  <si>
     <t>captivating</t>
   </si>
   <si>
-    <t>comforted</t>
+    <t>disconcerting</t>
+  </si>
+  <si>
+    <t>dreaded</t>
+  </si>
+  <si>
+    <t>embarrassed</t>
+  </si>
+  <si>
+    <t>emotion</t>
+  </si>
+  <si>
+    <t>exhilarated</t>
+  </si>
+  <si>
+    <t>frustrated</t>
+  </si>
+  <si>
+    <t>giddy</t>
+  </si>
+  <si>
+    <t>hungry</t>
+  </si>
+  <si>
+    <t>irritated</t>
+  </si>
+  <si>
+    <t>irritating</t>
+  </si>
+  <si>
+    <t>nasty</t>
+  </si>
+  <si>
+    <t>ominous</t>
+  </si>
+  <si>
+    <t>peacefulness</t>
+  </si>
+  <si>
+    <t>phobia</t>
+  </si>
+  <si>
+    <t>profound</t>
+  </si>
+  <si>
+    <t>regretting</t>
+  </si>
+  <si>
+    <t>screaming</t>
+  </si>
+  <si>
+    <t>spellbinding</t>
+  </si>
+  <si>
+    <t>spellbound</t>
+  </si>
+  <si>
+    <t>stoked</t>
+  </si>
+  <si>
+    <t>subtle</t>
+  </si>
+  <si>
+    <t>suprised</t>
+  </si>
+  <si>
+    <t>thrills</t>
+  </si>
+  <si>
+    <t>tranquil</t>
+  </si>
+  <si>
+    <t>tranquility</t>
+  </si>
+  <si>
+    <t>underwhelmed</t>
+  </si>
+  <si>
+    <t>unfair</t>
+  </si>
+  <si>
+    <t>unfriendly</t>
+  </si>
+  <si>
+    <t>unnerving</t>
+  </si>
+  <si>
+    <t>wicked</t>
+  </si>
+  <si>
+    <t>wildest</t>
+  </si>
+  <si>
+    <t>aggressively</t>
+  </si>
+  <si>
+    <t>ambivalent</t>
+  </si>
+  <si>
+    <t>apprehensions</t>
+  </si>
+  <si>
+    <t>aprehensive</t>
+  </si>
+  <si>
+    <t>astonished</t>
+  </si>
+  <si>
+    <t>astounded</t>
+  </si>
+  <si>
+    <t>beneficial</t>
+  </si>
+  <si>
+    <t>candid</t>
+  </si>
+  <si>
+    <t>carefree</t>
+  </si>
+  <si>
+    <t>cheer</t>
+  </si>
+  <si>
+    <t>compassion</t>
+  </si>
+  <si>
+    <t>compassionate</t>
+  </si>
+  <si>
+    <t>curiosity</t>
   </si>
   <si>
     <t>daunting</t>
   </si>
   <si>
-    <t>envy</t>
-  </si>
-  <si>
-    <t>faultless</t>
-  </si>
-  <si>
-    <t>gloomy</t>
+    <t>dazzled</t>
+  </si>
+  <si>
+    <t>deaf</t>
+  </si>
+  <si>
+    <t>dreaming</t>
+  </si>
+  <si>
+    <t>ecstasy</t>
+  </si>
+  <si>
+    <t>guilty</t>
+  </si>
+  <si>
+    <t>happiness</t>
   </si>
   <si>
     <t>harrowing</t>
   </si>
   <si>
-    <t>hated</t>
-  </si>
-  <si>
-    <t>hates</t>
-  </si>
-  <si>
-    <t>intimidating</t>
-  </si>
-  <si>
-    <t>jitters</t>
-  </si>
-  <si>
-    <t>joyful</t>
-  </si>
-  <si>
-    <t>luscious</t>
-  </si>
-  <si>
-    <t>marveled</t>
-  </si>
-  <si>
-    <t>nauseated</t>
-  </si>
-  <si>
-    <t>overwhelmingly</t>
-  </si>
-  <si>
-    <t>pity</t>
-  </si>
-  <si>
-    <t>scare</t>
-  </si>
-  <si>
-    <t>shock</t>
-  </si>
-  <si>
-    <t>stressful</t>
-  </si>
-  <si>
-    <t>suprise</t>
-  </si>
-  <si>
-    <t>wowed</t>
-  </si>
-  <si>
-    <t>disconcerting</t>
-  </si>
-  <si>
-    <t>dreaded</t>
-  </si>
-  <si>
-    <t>embarrassed</t>
-  </si>
-  <si>
-    <t>emotion</t>
-  </si>
-  <si>
-    <t>exhilarated</t>
-  </si>
-  <si>
-    <t>frustrated</t>
-  </si>
-  <si>
-    <t>giddy</t>
-  </si>
-  <si>
-    <t>hungry</t>
-  </si>
-  <si>
-    <t>irritated</t>
-  </si>
-  <si>
-    <t>irritating</t>
-  </si>
-  <si>
-    <t>nasty</t>
-  </si>
-  <si>
-    <t>ominous</t>
-  </si>
-  <si>
-    <t>peacefulness</t>
-  </si>
-  <si>
-    <t>phobia</t>
-  </si>
-  <si>
-    <t>profound</t>
-  </si>
-  <si>
-    <t>regretting</t>
-  </si>
-  <si>
-    <t>screaming</t>
-  </si>
-  <si>
-    <t>spellbinding</t>
-  </si>
-  <si>
-    <t>spellbound</t>
-  </si>
-  <si>
-    <t>stoked</t>
-  </si>
-  <si>
-    <t>subtle</t>
-  </si>
-  <si>
-    <t>suprised</t>
-  </si>
-  <si>
-    <t>thrills</t>
-  </si>
-  <si>
-    <t>tranquil</t>
-  </si>
-  <si>
-    <t>tranquility</t>
-  </si>
-  <si>
-    <t>underwhelmed</t>
-  </si>
-  <si>
-    <t>unfair</t>
-  </si>
-  <si>
-    <t>unfriendly</t>
-  </si>
-  <si>
-    <t>unnerving</t>
-  </si>
-  <si>
-    <t>wicked</t>
-  </si>
-  <si>
-    <t>wildest</t>
-  </si>
-  <si>
-    <t>aggressively</t>
-  </si>
-  <si>
-    <t>ambivalent</t>
-  </si>
-  <si>
-    <t>apprehensions</t>
-  </si>
-  <si>
-    <t>aprehensive</t>
-  </si>
-  <si>
-    <t>astonished</t>
-  </si>
-  <si>
-    <t>astounded</t>
-  </si>
-  <si>
-    <t>beneficial</t>
-  </si>
-  <si>
-    <t>candid</t>
-  </si>
-  <si>
-    <t>carefree</t>
-  </si>
-  <si>
-    <t>cheer</t>
-  </si>
-  <si>
-    <t>compassion</t>
-  </si>
-  <si>
-    <t>compassionate</t>
-  </si>
-  <si>
-    <t>curiosity</t>
-  </si>
-  <si>
-    <t>dazzled</t>
-  </si>
-  <si>
-    <t>deaf</t>
-  </si>
-  <si>
-    <t>dreaming</t>
-  </si>
-  <si>
-    <t>ecstasy</t>
-  </si>
-  <si>
-    <t>guilty</t>
-  </si>
-  <si>
-    <t>happiness</t>
-  </si>
-  <si>
     <t>heartfelt</t>
   </si>
   <si>
@@ -3295,222 +3295,222 @@
     <t>忧虑 / 疑虑不安</t>
   </si>
   <si>
+    <t>感到安慰安心的</t>
+  </si>
+  <si>
+    <t>羡慕 / 嫉妒</t>
+  </si>
+  <si>
+    <t>无可挑剔完美的</t>
+  </si>
+  <si>
+    <t>阴沉的 / 沮丧的</t>
+  </si>
+  <si>
+    <t>讨厌 / 极为憎恶的</t>
+  </si>
+  <si>
+    <t>厌恶 / 讨厌</t>
+  </si>
+  <si>
+    <t>令人胆怯令人畏惧的</t>
+  </si>
+  <si>
+    <t>忐忑不安 / 紧张发抖感</t>
+  </si>
+  <si>
+    <t>充满喜悦欢快的</t>
+  </si>
+  <si>
+    <t>秀美令人心旷神怡的</t>
+  </si>
+  <si>
+    <t>惊叹赞赏的</t>
+  </si>
+  <si>
+    <t>感到恶心反胃不适的</t>
+  </si>
+  <si>
+    <t>压倒性震撼地</t>
+  </si>
+  <si>
+    <t>遗憾 / 同情怜悯</t>
+  </si>
+  <si>
+    <t>吓人 / 引发恐慌的</t>
+  </si>
+  <si>
+    <t>震惊 / 冲击</t>
+  </si>
+  <si>
+    <t>令人压力重重焦虑的（Stress/Anxiety State）</t>
+  </si>
+  <si>
+    <t>惊喜 / 意料之外（错别字变体）</t>
+  </si>
+  <si>
+    <t>被深深惊叹震撼的</t>
+  </si>
+  <si>
     <t>扣人心弦引人入胜的</t>
   </si>
   <si>
-    <t>感到安慰安心的</t>
+    <t>令人不安的</t>
+  </si>
+  <si>
+    <t>令人害怕恐惧的 / 提心吊胆</t>
+  </si>
+  <si>
+    <t>感到尴尬难堪的</t>
+  </si>
+  <si>
+    <t>情感 / 情绪</t>
+  </si>
+  <si>
+    <t>感到无比兴奋酣畅的</t>
+  </si>
+  <si>
+    <t>感到沮丧的 / 挫败的</t>
+  </si>
+  <si>
+    <t>兴奋得头晕目眩欢欣的</t>
+  </si>
+  <si>
+    <t>贪婪的（money hungry）</t>
+  </si>
+  <si>
+    <t>感到恼火烦躁的</t>
+  </si>
+  <si>
+    <t>令人烦躁恼火的</t>
+  </si>
+  <si>
+    <t>令人厌恶的 / 恶劣的</t>
+  </si>
+  <si>
+    <t>不详的 / 不妙的</t>
+  </si>
+  <si>
+    <t>宁静详和感</t>
+  </si>
+  <si>
+    <t>恐惧症 / 恐高心理</t>
+  </si>
+  <si>
+    <t>深刻震撼的</t>
+  </si>
+  <si>
+    <t>感到后悔遗憾的</t>
+  </si>
+  <si>
+    <t>惊恐尖叫的</t>
+  </si>
+  <si>
+    <t>扣人心弦迷人的</t>
+  </si>
+  <si>
+    <t>出神为之入迷的</t>
+  </si>
+  <si>
+    <t>极为激动期待的</t>
+  </si>
+  <si>
+    <t>微妙精细的</t>
+  </si>
+  <si>
+    <t>感到惊喜惊讶的（错别字变体）</t>
+  </si>
+  <si>
+    <t>刺激 / 快感</t>
+  </si>
+  <si>
+    <t>清幽宁静的（Calmness/Serenity State）</t>
+  </si>
+  <si>
+    <t>宁静 / 平和</t>
+  </si>
+  <si>
+    <t>大失所望未达预期的</t>
+  </si>
+  <si>
+    <t>不公平的 / 冤枉的</t>
+  </si>
+  <si>
+    <t>不友善的</t>
+  </si>
+  <si>
+    <t>令人发慌不安吓人的</t>
+  </si>
+  <si>
+    <t>太棒了 / 绝妙的</t>
+  </si>
+  <si>
+    <t>最疯狂的（狂想）</t>
+  </si>
+  <si>
+    <t>挑衅攻击地 / 极其恶劣地</t>
+  </si>
+  <si>
+    <t>矛盾复杂心理的</t>
+  </si>
+  <si>
+    <t>顾虑 / 忧虑不安</t>
+  </si>
+  <si>
+    <t>感到忧虑不安的（错别字变体）</t>
+  </si>
+  <si>
+    <t>感到十分惊异惊叹的</t>
+  </si>
+  <si>
+    <t>感到十分震惊震撼的</t>
+  </si>
+  <si>
+    <t>有益的 / 有帮助的</t>
+  </si>
+  <si>
+    <t>坦率真诚的</t>
+  </si>
+  <si>
+    <t>无忧无虑自在的</t>
+  </si>
+  <si>
+    <t>振奋 / 欢呼</t>
+  </si>
+  <si>
+    <t>同理心 / 关切</t>
+  </si>
+  <si>
+    <t>富有同理心体贴的</t>
+  </si>
+  <si>
+    <t>好奇心 / 探索欲</t>
   </si>
   <si>
     <t>令人望而生畏胆怯的</t>
   </si>
   <si>
-    <t>羡慕 / 嫉妒</t>
-  </si>
-  <si>
-    <t>无可挑剔完美的</t>
-  </si>
-  <si>
-    <t>阴沉的 / 沮丧的</t>
+    <t>目眩神迷震撼的</t>
+  </si>
+  <si>
+    <t>听而不闻冷漠的（fell on deaf ears）</t>
+  </si>
+  <si>
+    <t>梦寐以求 / 心驰神往</t>
+  </si>
+  <si>
+    <t>狂喜 / 极乐状态</t>
+  </si>
+  <si>
+    <t>内疚内疚感</t>
+  </si>
+  <si>
+    <t>幸福快乐感</t>
   </si>
   <si>
     <t>令人触目惊心惊恐的</t>
   </si>
   <si>
-    <t>讨厌 / 极为憎恶的</t>
-  </si>
-  <si>
-    <t>厌恶 / 讨厌</t>
-  </si>
-  <si>
-    <t>令人胆怯令人畏惧的</t>
-  </si>
-  <si>
-    <t>忐忑不安 / 紧张发抖感</t>
-  </si>
-  <si>
-    <t>充满喜悦欢快的</t>
-  </si>
-  <si>
-    <t>秀美令人心旷神怡的</t>
-  </si>
-  <si>
-    <t>惊叹赞赏的</t>
-  </si>
-  <si>
-    <t>感到恶心反胃不适的</t>
-  </si>
-  <si>
-    <t>压倒性震撼地</t>
-  </si>
-  <si>
-    <t>遗憾 / 同情怜悯</t>
-  </si>
-  <si>
-    <t>吓人 / 引发恐慌的</t>
-  </si>
-  <si>
-    <t>震惊 / 冲击</t>
-  </si>
-  <si>
-    <t>令人压力重重焦虑的（Stress/Anxiety State）</t>
-  </si>
-  <si>
-    <t>惊喜 / 意料之外（错别字变体）</t>
-  </si>
-  <si>
-    <t>被深深惊叹震撼的</t>
-  </si>
-  <si>
-    <t>令人不安的</t>
-  </si>
-  <si>
-    <t>令人害怕恐惧的 / 提心吊胆</t>
-  </si>
-  <si>
-    <t>感到尴尬难堪的</t>
-  </si>
-  <si>
-    <t>情感 / 情绪</t>
-  </si>
-  <si>
-    <t>感到无比兴奋酣畅的</t>
-  </si>
-  <si>
-    <t>感到沮丧的 / 挫败的</t>
-  </si>
-  <si>
-    <t>兴奋得头晕目眩欢欣的</t>
-  </si>
-  <si>
-    <t>贪婪的（money hungry）</t>
-  </si>
-  <si>
-    <t>感到恼火烦躁的</t>
-  </si>
-  <si>
-    <t>令人烦躁恼火的</t>
-  </si>
-  <si>
-    <t>令人厌恶的 / 恶劣的</t>
-  </si>
-  <si>
-    <t>不详的 / 不妙的</t>
-  </si>
-  <si>
-    <t>宁静详和感</t>
-  </si>
-  <si>
-    <t>恐惧症 / 恐高心理</t>
-  </si>
-  <si>
-    <t>深刻震撼的</t>
-  </si>
-  <si>
-    <t>感到后悔遗憾的</t>
-  </si>
-  <si>
-    <t>惊恐尖叫的</t>
-  </si>
-  <si>
-    <t>扣人心弦迷人的</t>
-  </si>
-  <si>
-    <t>出神为之入迷的</t>
-  </si>
-  <si>
-    <t>极为激动期待的</t>
-  </si>
-  <si>
-    <t>微妙精细的</t>
-  </si>
-  <si>
-    <t>感到惊喜惊讶的（错别字变体）</t>
-  </si>
-  <si>
-    <t>刺激 / 快感</t>
-  </si>
-  <si>
-    <t>清幽宁静的（Calmness/Serenity State）</t>
-  </si>
-  <si>
-    <t>宁静 / 平和</t>
-  </si>
-  <si>
-    <t>大失所望未达预期的</t>
-  </si>
-  <si>
-    <t>不公平的 / 冤枉的</t>
-  </si>
-  <si>
-    <t>不友善的</t>
-  </si>
-  <si>
-    <t>令人发慌不安吓人的</t>
-  </si>
-  <si>
-    <t>太棒了 / 绝妙的</t>
-  </si>
-  <si>
-    <t>最疯狂的（狂想）</t>
-  </si>
-  <si>
-    <t>挑衅攻击地 / 极其恶劣地</t>
-  </si>
-  <si>
-    <t>矛盾复杂心理的</t>
-  </si>
-  <si>
-    <t>顾虑 / 忧虑不安</t>
-  </si>
-  <si>
-    <t>感到忧虑不安的（错别字变体）</t>
-  </si>
-  <si>
-    <t>感到十分惊异惊叹的</t>
-  </si>
-  <si>
-    <t>感到十分震惊震撼的</t>
-  </si>
-  <si>
-    <t>有益的 / 有帮助的</t>
-  </si>
-  <si>
-    <t>坦率真诚的</t>
-  </si>
-  <si>
-    <t>无忧无虑自在的</t>
-  </si>
-  <si>
-    <t>振奋 / 欢呼</t>
-  </si>
-  <si>
-    <t>同理心 / 关切</t>
-  </si>
-  <si>
-    <t>富有同理心体贴的</t>
-  </si>
-  <si>
-    <t>好奇心 / 探索欲</t>
-  </si>
-  <si>
-    <t>目眩神迷震撼的</t>
-  </si>
-  <si>
-    <t>听而不闻冷漠的（fell on deaf ears）</t>
-  </si>
-  <si>
-    <t>梦寐以求 / 心驰神往</t>
-  </si>
-  <si>
-    <t>狂喜 / 极乐状态</t>
-  </si>
-  <si>
-    <t>内疚内疚感</t>
-  </si>
-  <si>
-    <t>幸福快乐感</t>
-  </si>
-  <si>
     <t>真挚的 / 出自内心的</t>
   </si>
   <si>
@@ -3736,25 +3736,25 @@
     <t>Envy</t>
   </si>
   <si>
+    <t>Anger / Dislike</t>
+  </si>
+  <si>
+    <t>Nervousness / Anxiety</t>
+  </si>
+  <si>
+    <t>Wonder / Awe</t>
+  </si>
+  <si>
+    <t>Pity / Sadness</t>
+  </si>
+  <si>
+    <t>Surprise</t>
+  </si>
+  <si>
+    <t>Amazement / Awe</t>
+  </si>
+  <si>
     <t>Fear / Dread</t>
-  </si>
-  <si>
-    <t>Anger / Dislike</t>
-  </si>
-  <si>
-    <t>Nervousness / Anxiety</t>
-  </si>
-  <si>
-    <t>Wonder / Awe</t>
-  </si>
-  <si>
-    <t>Pity / Sadness</t>
-  </si>
-  <si>
-    <t>Surprise</t>
-  </si>
-  <si>
-    <t>Amazement / Awe</t>
   </si>
   <si>
     <t>Excitement / Joy</t>
@@ -4956,12 +4956,6 @@
     <t>review_c542b91f8f33b62598c7e8e7 :: The whole experience was fabulous from the convenience of short notice booking to the easy check in and ultimately with the flight and our pilot! The facility is welcoming and the ...</t>
   </si>
   <si>
-    <t>Review context: captivating</t>
-  </si>
-  <si>
-    <t>Review context: daunting</t>
-  </si>
-  <si>
     <t>review_1414273dd7063c526a44d117 :: This was one of lifetime plane trip realy memorable. I simply envy pilots they get to do this and get paid for it. Just seeing the wonderful mountain range up close is breathtaking...</t>
   </si>
   <si>
@@ -4971,9 +4965,6 @@
     <t>review_a49c3b4b417661efc807e243 :: Well, there really is a reason that this is rated number 1 for attractions and activities...there really is no downside.  Firstly, making a reservation by phone or online via their...</t>
   </si>
   <si>
-    <t>Review context: harrowing</t>
-  </si>
-  <si>
     <t>review_5fe9fad9238c2de93e358451 :: I had a "reservation" to fly, but waited over a hour. I saw lightening and storm clouds- I was told by pilot that it was a small cell that we'd fly around. IMMEDIATELY after takeof...</t>
   </si>
   <si>
@@ -5017,6 +5008,9 @@
   </si>
   <si>
     <t>review_5035b0fc89c249531e5a177f :: My family and I toured with K2 on a day that didn't have great weather. We were supposed to have a flightseeing tour and glacier landing at 1 pm, but because the weather was poor, ...</t>
+  </si>
+  <si>
+    <t>review_e64fadc568774df30ea12ccb :: Our pilot, Rosemarie, provided a wonderful flight and narration.   She was consistently focused on meeting our needs, answering questions with insightful responses, and proactively...</t>
   </si>
   <si>
     <t>review_b70a4a0ae56a29332a7fd7e6 :: We took Friday Harbor Seaplanes to and from Renton/San Juan Island. The flight was on time and the pilots seemed knowledgeable. Scenery was fantastic. My only complaint is that bot...</t>
@@ -5144,6 +5138,9 @@
   </si>
   <si>
     <t>review_a485c5e820c7e55c86de9a0b :: We decided on a whim to do a plane tour of Maui. WOW did we pick the right guy. The plane was as smooth as the operator. Absolutely flawless. We have done a ton of things so far on...</t>
+  </si>
+  <si>
+    <t>review_b7f01c12e058877205debe1a :: This was a great experience from start to finish, starting with quick responses to initial enquiries, preflight contacts and information, safety briefing and the engagement of an e...</t>
   </si>
   <si>
     <t>review_61a9d3d1fdbcd064bf4345ca :: We had an amazing Denali experience with Matt as our wonderful pilot!  Staff at the facility were very helpful and friendly making sure we knew what to do prior to boarding aircraf...</t>
@@ -19571,13 +19568,13 @@
         <v>1093</v>
       </c>
       <c r="D480" t="s">
-        <v>1225</v>
+        <v>1238</v>
       </c>
       <c r="E480" t="s">
-        <v>1261</v>
+        <v>1264</v>
       </c>
       <c r="F480" t="s">
-        <v>1269</v>
+        <v>1266</v>
       </c>
       <c r="G480">
         <v>5</v>
@@ -19586,7 +19583,7 @@
         <v>5</v>
       </c>
       <c r="I480" t="s">
-        <v>1630</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="481" spans="1:9">
@@ -19600,7 +19597,7 @@
         <v>1094</v>
       </c>
       <c r="D481" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="E481" t="s">
         <v>1264</v>
@@ -19615,7 +19612,7 @@
         <v>5</v>
       </c>
       <c r="I481" t="s">
-        <v>1288</v>
+        <v>1630</v>
       </c>
     </row>
     <row r="482" spans="1:9">
@@ -19629,13 +19626,13 @@
         <v>1095</v>
       </c>
       <c r="D482" t="s">
-        <v>1227</v>
+        <v>1221</v>
       </c>
       <c r="E482" t="s">
         <v>1261</v>
       </c>
       <c r="F482" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="G482">
         <v>5</v>
@@ -19658,19 +19655,19 @@
         <v>1096</v>
       </c>
       <c r="D483" t="s">
-        <v>1239</v>
+        <v>1221</v>
       </c>
       <c r="E483" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="F483" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="G483">
         <v>5</v>
       </c>
       <c r="H483">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I483" t="s">
         <v>1632</v>
@@ -19681,19 +19678,19 @@
         <v>491</v>
       </c>
       <c r="B484" t="s">
-        <v>491</v>
+        <v>618</v>
       </c>
       <c r="C484" t="s">
         <v>1097</v>
       </c>
       <c r="D484" t="s">
-        <v>1221</v>
+        <v>1240</v>
       </c>
       <c r="E484" t="s">
-        <v>1261</v>
+        <v>1264</v>
       </c>
       <c r="F484" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="G484">
         <v>5</v>
@@ -19710,25 +19707,25 @@
         <v>492</v>
       </c>
       <c r="B485" t="s">
-        <v>492</v>
+        <v>618</v>
       </c>
       <c r="C485" t="s">
         <v>1098</v>
       </c>
       <c r="D485" t="s">
-        <v>1221</v>
+        <v>1240</v>
       </c>
       <c r="E485" t="s">
-        <v>1262</v>
+        <v>1264</v>
       </c>
       <c r="F485" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="G485">
         <v>5</v>
       </c>
       <c r="H485">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I485" t="s">
         <v>1634</v>
@@ -19745,13 +19742,13 @@
         <v>1099</v>
       </c>
       <c r="D486" t="s">
-        <v>1240</v>
+        <v>1221</v>
       </c>
       <c r="E486" t="s">
         <v>1261</v>
       </c>
       <c r="F486" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="G486">
         <v>5</v>
@@ -19768,7 +19765,7 @@
         <v>494</v>
       </c>
       <c r="B487" t="s">
-        <v>618</v>
+        <v>494</v>
       </c>
       <c r="C487" t="s">
         <v>1100</v>
@@ -19797,19 +19794,19 @@
         <v>495</v>
       </c>
       <c r="B488" t="s">
-        <v>618</v>
+        <v>495</v>
       </c>
       <c r="C488" t="s">
         <v>1101</v>
       </c>
       <c r="D488" t="s">
-        <v>1241</v>
+        <v>1221</v>
       </c>
       <c r="E488" t="s">
         <v>1264</v>
       </c>
       <c r="F488" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="G488">
         <v>5</v>
@@ -19855,7 +19852,7 @@
         <v>497</v>
       </c>
       <c r="B490" t="s">
-        <v>497</v>
+        <v>619</v>
       </c>
       <c r="C490" t="s">
         <v>1103</v>
@@ -19942,7 +19939,7 @@
         <v>500</v>
       </c>
       <c r="B493" t="s">
-        <v>619</v>
+        <v>500</v>
       </c>
       <c r="C493" t="s">
         <v>1106</v>
@@ -19980,7 +19977,7 @@
         <v>1221</v>
       </c>
       <c r="E494" t="s">
-        <v>1264</v>
+        <v>1261</v>
       </c>
       <c r="F494" t="s">
         <v>1267</v>
@@ -20006,13 +20003,13 @@
         <v>1108</v>
       </c>
       <c r="D495" t="s">
-        <v>1221</v>
+        <v>1230</v>
       </c>
       <c r="E495" t="s">
-        <v>1261</v>
+        <v>1264</v>
       </c>
       <c r="F495" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="G495">
         <v>5</v>
@@ -20035,13 +20032,13 @@
         <v>1109</v>
       </c>
       <c r="D496" t="s">
-        <v>1244</v>
+        <v>1221</v>
       </c>
       <c r="E496" t="s">
         <v>1264</v>
       </c>
       <c r="F496" t="s">
-        <v>1266</v>
+        <v>1268</v>
       </c>
       <c r="G496">
         <v>5</v>
@@ -20058,19 +20055,19 @@
         <v>504</v>
       </c>
       <c r="B497" t="s">
-        <v>504</v>
+        <v>76</v>
       </c>
       <c r="C497" t="s">
         <v>1110</v>
       </c>
       <c r="D497" t="s">
-        <v>1221</v>
+        <v>1244</v>
       </c>
       <c r="E497" t="s">
-        <v>1261</v>
+        <v>1264</v>
       </c>
       <c r="F497" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="G497">
         <v>5</v>
@@ -20093,7 +20090,7 @@
         <v>1111</v>
       </c>
       <c r="D498" t="s">
-        <v>1230</v>
+        <v>1245</v>
       </c>
       <c r="E498" t="s">
         <v>1264</v>
@@ -20122,19 +20119,19 @@
         <v>1112</v>
       </c>
       <c r="D499" t="s">
-        <v>1221</v>
+        <v>1225</v>
       </c>
       <c r="E499" t="s">
-        <v>1264</v>
+        <v>1261</v>
       </c>
       <c r="F499" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="G499">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H499">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I499" t="s">
         <v>1648</v>
@@ -20145,25 +20142,25 @@
         <v>507</v>
       </c>
       <c r="B500" t="s">
-        <v>76</v>
+        <v>507</v>
       </c>
       <c r="C500" t="s">
         <v>1113</v>
       </c>
       <c r="D500" t="s">
-        <v>1245</v>
+        <v>1221</v>
       </c>
       <c r="E500" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="F500" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="G500">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H500">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I500" t="s">
         <v>1649</v>
@@ -20174,7 +20171,7 @@
         <v>508</v>
       </c>
       <c r="B501" t="s">
-        <v>508</v>
+        <v>620</v>
       </c>
       <c r="C501" t="s">
         <v>1114</v>
@@ -20189,10 +20186,10 @@
         <v>1266</v>
       </c>
       <c r="G501">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H501">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I501" t="s">
         <v>1650</v>
@@ -20212,10 +20209,10 @@
         <v>1221</v>
       </c>
       <c r="E502" t="s">
-        <v>1262</v>
+        <v>1264</v>
       </c>
       <c r="F502" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
       <c r="G502">
         <v>4</v>
@@ -20232,19 +20229,19 @@
         <v>510</v>
       </c>
       <c r="B503" t="s">
-        <v>620</v>
+        <v>510</v>
       </c>
       <c r="C503" t="s">
         <v>1116</v>
       </c>
       <c r="D503" t="s">
-        <v>1240</v>
+        <v>1221</v>
       </c>
       <c r="E503" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="F503" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="G503">
         <v>4</v>
@@ -20267,13 +20264,13 @@
         <v>1117</v>
       </c>
       <c r="D504" t="s">
-        <v>1221</v>
+        <v>1247</v>
       </c>
       <c r="E504" t="s">
         <v>1264</v>
       </c>
       <c r="F504" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="G504">
         <v>4</v>
@@ -20299,7 +20296,7 @@
         <v>1221</v>
       </c>
       <c r="E505" t="s">
-        <v>1262</v>
+        <v>1264</v>
       </c>
       <c r="F505" t="s">
         <v>1265</v>
@@ -20357,7 +20354,7 @@
         <v>1221</v>
       </c>
       <c r="E507" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="F507" t="s">
         <v>1265</v>
@@ -20383,13 +20380,13 @@
         <v>1121</v>
       </c>
       <c r="D508" t="s">
-        <v>1247</v>
+        <v>1221</v>
       </c>
       <c r="E508" t="s">
         <v>1264</v>
       </c>
       <c r="F508" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="G508">
         <v>4</v>
@@ -20412,13 +20409,13 @@
         <v>1122</v>
       </c>
       <c r="D509" t="s">
-        <v>1221</v>
+        <v>1248</v>
       </c>
       <c r="E509" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="F509" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="G509">
         <v>4</v>
@@ -20444,16 +20441,16 @@
         <v>1221</v>
       </c>
       <c r="E510" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="F510" t="s">
-        <v>1267</v>
+        <v>1265</v>
       </c>
       <c r="G510">
         <v>4</v>
       </c>
       <c r="H510">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I510" t="s">
         <v>1659</v>
@@ -20470,19 +20467,19 @@
         <v>1124</v>
       </c>
       <c r="D511" t="s">
-        <v>1248</v>
+        <v>1221</v>
       </c>
       <c r="E511" t="s">
-        <v>1261</v>
+        <v>1262</v>
       </c>
       <c r="F511" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="G511">
         <v>4</v>
       </c>
       <c r="H511">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I511" t="s">
         <v>1660</v>
@@ -20499,19 +20496,19 @@
         <v>1125</v>
       </c>
       <c r="D512" t="s">
-        <v>1221</v>
+        <v>1249</v>
       </c>
       <c r="E512" t="s">
-        <v>1262</v>
+        <v>1264</v>
       </c>
       <c r="F512" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="G512">
         <v>4</v>
       </c>
       <c r="H512">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I512" t="s">
         <v>1661</v>
@@ -20528,13 +20525,13 @@
         <v>1126</v>
       </c>
       <c r="D513" t="s">
-        <v>1221</v>
+        <v>1229</v>
       </c>
       <c r="E513" t="s">
-        <v>1262</v>
+        <v>1264</v>
       </c>
       <c r="F513" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="G513">
         <v>4</v>
@@ -20557,13 +20554,13 @@
         <v>1127</v>
       </c>
       <c r="D514" t="s">
-        <v>1249</v>
+        <v>1221</v>
       </c>
       <c r="E514" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="F514" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="G514">
         <v>4</v>
@@ -20580,13 +20577,13 @@
         <v>522</v>
       </c>
       <c r="B515" t="s">
-        <v>522</v>
+        <v>621</v>
       </c>
       <c r="C515" t="s">
         <v>1128</v>
       </c>
       <c r="D515" t="s">
-        <v>1229</v>
+        <v>1250</v>
       </c>
       <c r="E515" t="s">
         <v>1264</v>
@@ -20598,7 +20595,7 @@
         <v>4</v>
       </c>
       <c r="H515">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I515" t="s">
         <v>1664</v>
@@ -20618,10 +20615,10 @@
         <v>1221</v>
       </c>
       <c r="E516" t="s">
-        <v>1262</v>
+        <v>1264</v>
       </c>
       <c r="F516" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
       <c r="G516">
         <v>4</v>
@@ -20638,19 +20635,19 @@
         <v>524</v>
       </c>
       <c r="B517" t="s">
-        <v>621</v>
+        <v>524</v>
       </c>
       <c r="C517" t="s">
         <v>1130</v>
       </c>
       <c r="D517" t="s">
-        <v>1250</v>
+        <v>1221</v>
       </c>
       <c r="E517" t="s">
-        <v>1264</v>
+        <v>1261</v>
       </c>
       <c r="F517" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="G517">
         <v>4</v>
@@ -20673,13 +20670,13 @@
         <v>1131</v>
       </c>
       <c r="D518" t="s">
-        <v>1221</v>
+        <v>1225</v>
       </c>
       <c r="E518" t="s">
         <v>1264</v>
       </c>
       <c r="F518" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="G518">
         <v>4</v>
@@ -20702,13 +20699,13 @@
         <v>1132</v>
       </c>
       <c r="D519" t="s">
-        <v>1221</v>
+        <v>1231</v>
       </c>
       <c r="E519" t="s">
-        <v>1261</v>
+        <v>1264</v>
       </c>
       <c r="F519" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="G519">
         <v>4</v>
@@ -20731,13 +20728,13 @@
         <v>1133</v>
       </c>
       <c r="D520" t="s">
-        <v>1225</v>
+        <v>1221</v>
       </c>
       <c r="E520" t="s">
-        <v>1264</v>
+        <v>1261</v>
       </c>
       <c r="F520" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="G520">
         <v>4</v>
@@ -20754,13 +20751,13 @@
         <v>528</v>
       </c>
       <c r="B521" t="s">
-        <v>528</v>
+        <v>75</v>
       </c>
       <c r="C521" t="s">
         <v>1134</v>
       </c>
       <c r="D521" t="s">
-        <v>1231</v>
+        <v>1244</v>
       </c>
       <c r="E521" t="s">
         <v>1264</v>
@@ -20792,10 +20789,10 @@
         <v>1221</v>
       </c>
       <c r="E522" t="s">
-        <v>1261</v>
+        <v>1262</v>
       </c>
       <c r="F522" t="s">
-        <v>1267</v>
+        <v>1265</v>
       </c>
       <c r="G522">
         <v>4</v>
@@ -20812,19 +20809,19 @@
         <v>530</v>
       </c>
       <c r="B523" t="s">
-        <v>75</v>
+        <v>530</v>
       </c>
       <c r="C523" t="s">
         <v>1136</v>
       </c>
       <c r="D523" t="s">
-        <v>1245</v>
+        <v>1221</v>
       </c>
       <c r="E523" t="s">
         <v>1264</v>
       </c>
       <c r="F523" t="s">
-        <v>1266</v>
+        <v>1268</v>
       </c>
       <c r="G523">
         <v>4</v>
@@ -20876,13 +20873,13 @@
         <v>1138</v>
       </c>
       <c r="D525" t="s">
-        <v>1221</v>
+        <v>1228</v>
       </c>
       <c r="E525" t="s">
         <v>1264</v>
       </c>
       <c r="F525" t="s">
-        <v>1268</v>
+        <v>1266</v>
       </c>
       <c r="G525">
         <v>4</v>
@@ -20891,7 +20888,7 @@
         <v>4</v>
       </c>
       <c r="I525" t="s">
-        <v>1674</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="526" spans="1:9">
@@ -20917,10 +20914,10 @@
         <v>4</v>
       </c>
       <c r="H526">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I526" t="s">
-        <v>1675</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="527" spans="1:9">
@@ -20934,13 +20931,13 @@
         <v>1140</v>
       </c>
       <c r="D527" t="s">
-        <v>1228</v>
+        <v>1221</v>
       </c>
       <c r="E527" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="F527" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="G527">
         <v>4</v>
@@ -20949,7 +20946,7 @@
         <v>4</v>
       </c>
       <c r="I527" t="s">
-        <v>1647</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="528" spans="1:9">
@@ -20966,19 +20963,19 @@
         <v>1221</v>
       </c>
       <c r="E528" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="F528" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
       <c r="G528">
         <v>4</v>
       </c>
       <c r="H528">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I528" t="s">
-        <v>1676</v>
+        <v>1617</v>
       </c>
     </row>
     <row r="529" spans="1:9">
@@ -20995,10 +20992,10 @@
         <v>1221</v>
       </c>
       <c r="E529" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="F529" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
       <c r="G529">
         <v>4</v>
@@ -21007,7 +21004,7 @@
         <v>4</v>
       </c>
       <c r="I529" t="s">
-        <v>1677</v>
+        <v>1676</v>
       </c>
     </row>
     <row r="530" spans="1:9">
@@ -21024,10 +21021,10 @@
         <v>1221</v>
       </c>
       <c r="E530" t="s">
-        <v>1261</v>
+        <v>1262</v>
       </c>
       <c r="F530" t="s">
-        <v>1267</v>
+        <v>1265</v>
       </c>
       <c r="G530">
         <v>4</v>
@@ -21036,7 +21033,7 @@
         <v>4</v>
       </c>
       <c r="I530" t="s">
-        <v>1617</v>
+        <v>1677</v>
       </c>
     </row>
     <row r="531" spans="1:9">
@@ -21053,19 +21050,19 @@
         <v>1221</v>
       </c>
       <c r="E531" t="s">
-        <v>1261</v>
+        <v>1262</v>
       </c>
       <c r="F531" t="s">
-        <v>1267</v>
+        <v>1265</v>
       </c>
       <c r="G531">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H531">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I531" t="s">
-        <v>1678</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="532" spans="1:9">
@@ -21079,22 +21076,22 @@
         <v>1145</v>
       </c>
       <c r="D532" t="s">
-        <v>1221</v>
+        <v>1251</v>
       </c>
       <c r="E532" t="s">
-        <v>1262</v>
+        <v>1264</v>
       </c>
       <c r="F532" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="G532">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H532">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I532" t="s">
-        <v>1679</v>
+        <v>1678</v>
       </c>
     </row>
     <row r="533" spans="1:9">
@@ -21102,19 +21099,19 @@
         <v>540</v>
       </c>
       <c r="B533" t="s">
-        <v>540</v>
+        <v>486</v>
       </c>
       <c r="C533" t="s">
         <v>1146</v>
       </c>
       <c r="D533" t="s">
-        <v>1221</v>
+        <v>1237</v>
       </c>
       <c r="E533" t="s">
-        <v>1262</v>
+        <v>1264</v>
       </c>
       <c r="F533" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="G533">
         <v>3</v>
@@ -21123,7 +21120,7 @@
         <v>3</v>
       </c>
       <c r="I533" t="s">
-        <v>1296</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="534" spans="1:9">
@@ -21131,13 +21128,13 @@
         <v>541</v>
       </c>
       <c r="B534" t="s">
-        <v>541</v>
+        <v>131</v>
       </c>
       <c r="C534" t="s">
         <v>1147</v>
       </c>
       <c r="D534" t="s">
-        <v>1251</v>
+        <v>1237</v>
       </c>
       <c r="E534" t="s">
         <v>1264</v>
@@ -21160,13 +21157,13 @@
         <v>542</v>
       </c>
       <c r="B535" t="s">
-        <v>486</v>
+        <v>542</v>
       </c>
       <c r="C535" t="s">
         <v>1148</v>
       </c>
       <c r="D535" t="s">
-        <v>1237</v>
+        <v>1252</v>
       </c>
       <c r="E535" t="s">
         <v>1264</v>
@@ -21189,13 +21186,13 @@
         <v>543</v>
       </c>
       <c r="B536" t="s">
-        <v>131</v>
+        <v>543</v>
       </c>
       <c r="C536" t="s">
         <v>1149</v>
       </c>
       <c r="D536" t="s">
-        <v>1237</v>
+        <v>1233</v>
       </c>
       <c r="E536" t="s">
         <v>1264</v>
@@ -21224,13 +21221,13 @@
         <v>1150</v>
       </c>
       <c r="D537" t="s">
-        <v>1252</v>
+        <v>1221</v>
       </c>
       <c r="E537" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="F537" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="G537">
         <v>3</v>
@@ -21253,13 +21250,13 @@
         <v>1151</v>
       </c>
       <c r="D538" t="s">
-        <v>1233</v>
+        <v>1221</v>
       </c>
       <c r="E538" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="F538" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="G538">
         <v>3</v>
@@ -21285,10 +21282,10 @@
         <v>1221</v>
       </c>
       <c r="E539" t="s">
-        <v>1262</v>
+        <v>1264</v>
       </c>
       <c r="F539" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
       <c r="G539">
         <v>3</v>
@@ -21340,13 +21337,13 @@
         <v>1154</v>
       </c>
       <c r="D541" t="s">
-        <v>1221</v>
+        <v>1253</v>
       </c>
       <c r="E541" t="s">
         <v>1264</v>
       </c>
       <c r="F541" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="G541">
         <v>3</v>
@@ -21369,13 +21366,13 @@
         <v>1155</v>
       </c>
       <c r="D542" t="s">
-        <v>1221</v>
+        <v>1253</v>
       </c>
       <c r="E542" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="F542" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="G542">
         <v>3</v>
@@ -21398,13 +21395,13 @@
         <v>1156</v>
       </c>
       <c r="D543" t="s">
-        <v>1253</v>
+        <v>1221</v>
       </c>
       <c r="E543" t="s">
         <v>1264</v>
       </c>
       <c r="F543" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="G543">
         <v>3</v>
@@ -21413,7 +21410,7 @@
         <v>3</v>
       </c>
       <c r="I543" t="s">
-        <v>1689</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="544" spans="1:9">
@@ -21427,13 +21424,13 @@
         <v>1157</v>
       </c>
       <c r="D544" t="s">
-        <v>1253</v>
+        <v>1227</v>
       </c>
       <c r="E544" t="s">
         <v>1261</v>
       </c>
       <c r="F544" t="s">
-        <v>1266</v>
+        <v>1269</v>
       </c>
       <c r="G544">
         <v>3</v>
@@ -21442,7 +21439,7 @@
         <v>3</v>
       </c>
       <c r="I544" t="s">
-        <v>1690</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="545" spans="1:9">
@@ -21456,13 +21453,13 @@
         <v>1158</v>
       </c>
       <c r="D545" t="s">
-        <v>1221</v>
+        <v>1245</v>
       </c>
       <c r="E545" t="s">
         <v>1264</v>
       </c>
       <c r="F545" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="G545">
         <v>3</v>
@@ -21471,7 +21468,7 @@
         <v>3</v>
       </c>
       <c r="I545" t="s">
-        <v>1290</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="546" spans="1:9">
@@ -21485,13 +21482,13 @@
         <v>1159</v>
       </c>
       <c r="D546" t="s">
-        <v>1246</v>
+        <v>1221</v>
       </c>
       <c r="E546" t="s">
-        <v>1264</v>
+        <v>1261</v>
       </c>
       <c r="F546" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="G546">
         <v>3</v>
@@ -21517,10 +21514,10 @@
         <v>1221</v>
       </c>
       <c r="E547" t="s">
-        <v>1261</v>
+        <v>1264</v>
       </c>
       <c r="F547" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
       <c r="G547">
         <v>3</v>
@@ -21543,13 +21540,13 @@
         <v>1161</v>
       </c>
       <c r="D548" t="s">
-        <v>1221</v>
+        <v>1254</v>
       </c>
       <c r="E548" t="s">
         <v>1264</v>
       </c>
       <c r="F548" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="G548">
         <v>3</v>
@@ -21558,7 +21555,7 @@
         <v>3</v>
       </c>
       <c r="I548" t="s">
-        <v>1693</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="549" spans="1:9">
@@ -21572,7 +21569,7 @@
         <v>1162</v>
       </c>
       <c r="D549" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="E549" t="s">
         <v>1264</v>
@@ -21587,7 +21584,7 @@
         <v>3</v>
       </c>
       <c r="I549" t="s">
-        <v>1486</v>
+        <v>1693</v>
       </c>
     </row>
     <row r="550" spans="1:9">
@@ -21601,13 +21598,13 @@
         <v>1163</v>
       </c>
       <c r="D550" t="s">
-        <v>1255</v>
+        <v>1221</v>
       </c>
       <c r="E550" t="s">
         <v>1264</v>
       </c>
       <c r="F550" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="G550">
         <v>3</v>
@@ -21630,13 +21627,13 @@
         <v>1164</v>
       </c>
       <c r="D551" t="s">
-        <v>1221</v>
+        <v>1246</v>
       </c>
       <c r="E551" t="s">
-        <v>1264</v>
+        <v>1261</v>
       </c>
       <c r="F551" t="s">
-        <v>1267</v>
+        <v>1269</v>
       </c>
       <c r="G551">
         <v>3</v>
@@ -21645,7 +21642,7 @@
         <v>3</v>
       </c>
       <c r="I551" t="s">
-        <v>1695</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="552" spans="1:9">
@@ -21674,7 +21671,7 @@
         <v>3</v>
       </c>
       <c r="I552" t="s">
-        <v>1696</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="553" spans="1:9">
@@ -21703,7 +21700,7 @@
         <v>3</v>
       </c>
       <c r="I553" t="s">
-        <v>1697</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="554" spans="1:9">
@@ -21732,7 +21729,7 @@
         <v>3</v>
       </c>
       <c r="I554" t="s">
-        <v>1698</v>
+        <v>1697</v>
       </c>
     </row>
     <row r="555" spans="1:9">
@@ -21761,7 +21758,7 @@
         <v>3</v>
       </c>
       <c r="I555" t="s">
-        <v>1699</v>
+        <v>1698</v>
       </c>
     </row>
     <row r="556" spans="1:9">
@@ -21819,7 +21816,7 @@
         <v>3</v>
       </c>
       <c r="I557" t="s">
-        <v>1700</v>
+        <v>1699</v>
       </c>
     </row>
     <row r="558" spans="1:9">
@@ -21848,7 +21845,7 @@
         <v>3</v>
       </c>
       <c r="I558" t="s">
-        <v>1701</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="559" spans="1:9">
@@ -21906,7 +21903,7 @@
         <v>3</v>
       </c>
       <c r="I560" t="s">
-        <v>1702</v>
+        <v>1701</v>
       </c>
     </row>
     <row r="561" spans="1:9">
@@ -21935,7 +21932,7 @@
         <v>3</v>
       </c>
       <c r="I561" t="s">
-        <v>1703</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="562" spans="1:9">
@@ -21993,7 +21990,7 @@
         <v>3</v>
       </c>
       <c r="I563" t="s">
-        <v>1704</v>
+        <v>1703</v>
       </c>
     </row>
     <row r="564" spans="1:9">
@@ -22022,7 +22019,7 @@
         <v>3</v>
       </c>
       <c r="I564" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
     </row>
     <row r="565" spans="1:9">
@@ -22051,7 +22048,7 @@
         <v>3</v>
       </c>
       <c r="I565" t="s">
-        <v>1706</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="566" spans="1:9">
@@ -22080,7 +22077,7 @@
         <v>3</v>
       </c>
       <c r="I566" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="567" spans="1:9">
@@ -22109,7 +22106,7 @@
         <v>2</v>
       </c>
       <c r="I567" t="s">
-        <v>1708</v>
+        <v>1707</v>
       </c>
     </row>
     <row r="568" spans="1:9">
@@ -22138,7 +22135,7 @@
         <v>2</v>
       </c>
       <c r="I568" t="s">
-        <v>1709</v>
+        <v>1708</v>
       </c>
     </row>
     <row r="569" spans="1:9">
@@ -22167,7 +22164,7 @@
         <v>2</v>
       </c>
       <c r="I569" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="570" spans="1:9">
@@ -22196,7 +22193,7 @@
         <v>2</v>
       </c>
       <c r="I570" t="s">
-        <v>1711</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="571" spans="1:9">
@@ -22225,7 +22222,7 @@
         <v>2</v>
       </c>
       <c r="I571" t="s">
-        <v>1712</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="572" spans="1:9">
@@ -22254,7 +22251,7 @@
         <v>2</v>
       </c>
       <c r="I572" t="s">
-        <v>1713</v>
+        <v>1712</v>
       </c>
     </row>
     <row r="573" spans="1:9">
@@ -22312,7 +22309,7 @@
         <v>2</v>
       </c>
       <c r="I574" t="s">
-        <v>1714</v>
+        <v>1713</v>
       </c>
     </row>
     <row r="575" spans="1:9">
@@ -22370,7 +22367,7 @@
         <v>2</v>
       </c>
       <c r="I576" t="s">
-        <v>1715</v>
+        <v>1714</v>
       </c>
     </row>
     <row r="577" spans="1:9">
@@ -22399,7 +22396,7 @@
         <v>2</v>
       </c>
       <c r="I577" t="s">
-        <v>1716</v>
+        <v>1715</v>
       </c>
     </row>
     <row r="578" spans="1:9">
@@ -22428,7 +22425,7 @@
         <v>1</v>
       </c>
       <c r="I578" t="s">
-        <v>1717</v>
+        <v>1716</v>
       </c>
     </row>
     <row r="579" spans="1:9">
@@ -22457,7 +22454,7 @@
         <v>2</v>
       </c>
       <c r="I579" t="s">
-        <v>1652</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="580" spans="1:9">
@@ -22486,7 +22483,7 @@
         <v>2</v>
       </c>
       <c r="I580" t="s">
-        <v>1718</v>
+        <v>1717</v>
       </c>
     </row>
     <row r="581" spans="1:9">
@@ -22515,7 +22512,7 @@
         <v>2</v>
       </c>
       <c r="I581" t="s">
-        <v>1719</v>
+        <v>1718</v>
       </c>
     </row>
     <row r="582" spans="1:9">
@@ -22544,7 +22541,7 @@
         <v>2</v>
       </c>
       <c r="I582" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
     </row>
     <row r="583" spans="1:9">
@@ -22573,7 +22570,7 @@
         <v>2</v>
       </c>
       <c r="I583" t="s">
-        <v>1721</v>
+        <v>1720</v>
       </c>
     </row>
     <row r="584" spans="1:9">
@@ -22602,7 +22599,7 @@
         <v>1</v>
       </c>
       <c r="I584" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
     </row>
     <row r="585" spans="1:9">
@@ -22631,7 +22628,7 @@
         <v>1</v>
       </c>
       <c r="I585" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="586" spans="1:9">
@@ -22660,7 +22657,7 @@
         <v>1</v>
       </c>
       <c r="I586" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
     </row>
     <row r="587" spans="1:9">
@@ -22689,7 +22686,7 @@
         <v>1</v>
       </c>
       <c r="I587" t="s">
-        <v>1661</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="588" spans="1:9">
@@ -22718,7 +22715,7 @@
         <v>1</v>
       </c>
       <c r="I588" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
     </row>
     <row r="589" spans="1:9">
@@ -22747,7 +22744,7 @@
         <v>1</v>
       </c>
       <c r="I589" t="s">
-        <v>1725</v>
+        <v>1724</v>
       </c>
     </row>
     <row r="590" spans="1:9">
@@ -22776,7 +22773,7 @@
         <v>1</v>
       </c>
       <c r="I590" t="s">
-        <v>1662</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="591" spans="1:9">
@@ -22805,7 +22802,7 @@
         <v>1</v>
       </c>
       <c r="I591" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
     </row>
     <row r="592" spans="1:9">
@@ -22834,7 +22831,7 @@
         <v>1</v>
       </c>
       <c r="I592" t="s">
-        <v>1727</v>
+        <v>1726</v>
       </c>
     </row>
     <row r="593" spans="1:9">
@@ -22863,7 +22860,7 @@
         <v>1</v>
       </c>
       <c r="I593" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
     </row>
     <row r="594" spans="1:9">
@@ -22892,7 +22889,7 @@
         <v>1</v>
       </c>
       <c r="I594" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
     </row>
     <row r="595" spans="1:9">
@@ -22921,7 +22918,7 @@
         <v>1</v>
       </c>
       <c r="I595" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="596" spans="1:9">
@@ -22950,7 +22947,7 @@
         <v>1</v>
       </c>
       <c r="I596" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
     </row>
     <row r="597" spans="1:9">
@@ -22979,7 +22976,7 @@
         <v>1</v>
       </c>
       <c r="I597" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
     </row>
     <row r="598" spans="1:9">
@@ -23037,7 +23034,7 @@
         <v>1</v>
       </c>
       <c r="I599" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
     </row>
     <row r="600" spans="1:9">
@@ -23066,7 +23063,7 @@
         <v>1</v>
       </c>
       <c r="I600" t="s">
-        <v>1734</v>
+        <v>1733</v>
       </c>
     </row>
     <row r="601" spans="1:9">
@@ -23077,7 +23074,7 @@
         <v>608</v>
       </c>
       <c r="C601" t="s">
-        <v>1118</v>
+        <v>1116</v>
       </c>
       <c r="D601" t="s">
         <v>1221</v>
@@ -23095,7 +23092,7 @@
         <v>1</v>
       </c>
       <c r="I601" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
     </row>
     <row r="602" spans="1:9">
@@ -23124,7 +23121,7 @@
         <v>1</v>
       </c>
       <c r="I602" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
     </row>
     <row r="603" spans="1:9">
@@ -23153,7 +23150,7 @@
         <v>1</v>
       </c>
       <c r="I603" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
     </row>
     <row r="604" spans="1:9">
@@ -23182,7 +23179,7 @@
         <v>1</v>
       </c>
       <c r="I604" t="s">
-        <v>1737</v>
+        <v>1736</v>
       </c>
     </row>
     <row r="605" spans="1:9">
@@ -23211,7 +23208,7 @@
         <v>1</v>
       </c>
       <c r="I605" t="s">
-        <v>1738</v>
+        <v>1737</v>
       </c>
     </row>
     <row r="606" spans="1:9">
@@ -23240,7 +23237,7 @@
         <v>1</v>
       </c>
       <c r="I606" t="s">
-        <v>1739</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="607" spans="1:9">
@@ -23269,7 +23266,7 @@
         <v>1</v>
       </c>
       <c r="I607" t="s">
-        <v>1740</v>
+        <v>1739</v>
       </c>
     </row>
     <row r="608" spans="1:9">
@@ -23298,7 +23295,7 @@
         <v>1</v>
       </c>
       <c r="I608" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
     </row>
     <row r="609" spans="1:9">
@@ -23327,7 +23324,7 @@
         <v>1</v>
       </c>
       <c r="I609" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
     </row>
   </sheetData>

</xml_diff>